<commit_message>
Matriz solo con número, línea y X: se quitan las columnas de texto y la matriz antigua con el texto en la columna D
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014C31pV7EjewnUgiuZ5eKhn
</commit_message>
<xml_diff>
--- a/taller/catalogo/v2/piloto_gpt-image/matriz_gpt-image.xlsx
+++ b/taller/catalogo/v2/piloto_gpt-image/matriz_gpt-image.xlsx
@@ -8,9 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="matriz" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="criterios" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="consultas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="columnas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="columnas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -57,7 +55,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -65,9 +63,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -434,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:TC86"/>
+  <dimension ref="A1:SY86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -956,10 +951,6 @@
     <col width="3.2" customWidth="1" min="517" max="517"/>
     <col width="3.2" customWidth="1" min="518" max="518"/>
     <col width="3.2" customWidth="1" min="519" max="519"/>
-    <col width="40" customWidth="1" min="520" max="520"/>
-    <col width="50" customWidth="1" min="521" max="521"/>
-    <col width="50" customWidth="1" min="522" max="522"/>
-    <col width="10" customWidth="1" min="523" max="523"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3840,26 +3831,6 @@
           <t>salida.validaciones</t>
         </is>
       </c>
-      <c r="SZ2" s="1" t="inlineStr">
-        <is>
-          <t>casos</t>
-        </is>
-      </c>
-      <c r="TA2" s="1" t="inlineStr">
-        <is>
-          <t>valor a insertar</t>
-        </is>
-      </c>
-      <c r="TB2" s="1" t="inlineStr">
-        <is>
-          <t>fundamento</t>
-        </is>
-      </c>
-      <c r="TC2" s="1" t="inlineStr">
-        <is>
-          <t>consulta</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3875,14 +3846,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ3" s="4" t="inlineStr"/>
-      <c r="TA3" s="4" t="inlineStr"/>
-      <c r="TB3" s="4" t="inlineStr">
-        <is>
-          <t>título del documento; delimita el alcance del archivo a GPT Image 2, no regula nada por sí</t>
-        </is>
-      </c>
-      <c r="TC3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5438,18 +5401,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ4" s="4" t="inlineStr"/>
-      <c r="TA4" s="4" t="inlineStr">
-        <is>
-          <t>gpt-image-2 por defecto en producción; gpt-image-1.5 y gpt-image-1 solo migración; gpt-image-1-mini económico</t>
-        </is>
-      </c>
-      <c r="TB4" s="4" t="inlineStr">
-        <is>
-          <t>«Production default OpenAI: gpt-image-2. Migration-only… Бюджетный: gpt-image-1-mini»</t>
-        </is>
-      </c>
-      <c r="TC4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5465,14 +5416,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ5" s="4" t="inlineStr"/>
-      <c r="TA5" s="4" t="inlineStr"/>
-      <c r="TB5" s="4" t="inlineStr">
-        <is>
-          <t>encabezado de sección «Estructura del prompt — 5 slots»; el contenido está en 002334–002336</t>
-        </is>
-      </c>
-      <c r="TC5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6998,18 +6941,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ6" s="4" t="inlineStr"/>
-      <c r="TA6" s="4" t="inlineStr">
-        <is>
-          <t>secciones con etiqueta, no texto corrido</t>
-        </is>
-      </c>
-      <c r="TB6" s="4" t="inlineStr">
-        <is>
-          <t>«Пиши лейблами, не сплошным текстом»: imperativo, vale para todo prompt de GPT Image 2</t>
-        </is>
-      </c>
-      <c r="TC6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8555,18 +8486,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ7" s="4" t="inlineStr"/>
-      <c r="TA7" s="4" t="inlineStr">
-        <is>
-          <t>Scene: location, time of day, background, environment / Subject: primary focus / Important Details: materials, textures, lighting, camera angle, mood, composition / Use Case: editorial, product mockup, UI, poster, infographic / Constraints: what must NOT change/appear</t>
-        </is>
-      </c>
-      <c r="TB7" s="4" t="inlineStr">
-        <is>
-          <t>bloque literal de los 5 slots bajo «Структура промпта — 5 slots»</t>
-        </is>
-      </c>
-      <c r="TC7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10097,18 +10016,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ8" s="4" t="inlineStr"/>
-      <c r="TA8" s="4" t="inlineStr">
-        <is>
-          <t>Constraints explícitas (el slot no puede ir vacío)</t>
-        </is>
-      </c>
-      <c r="TB8" s="4" t="inlineStr">
-        <is>
-          <t>«Без явных constraints модель дрейфует»: sin restricciones explícitas el modelo deriva</t>
-        </is>
-      </c>
-      <c r="TC8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -10124,14 +10031,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ9" s="4" t="inlineStr"/>
-      <c r="TA9" s="4" t="inlineStr"/>
-      <c r="TB9" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Ejemplo mínimo»; el ejemplo es 002338</t>
-        </is>
-      </c>
-      <c r="TC9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11657,18 +11556,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ10" s="4" t="inlineStr"/>
-      <c r="TA10" s="4" t="inlineStr">
-        <is>
-          <t>prompt del florista de Lisboa con los 5 slots completos</t>
-        </is>
-      </c>
-      <c r="TB10" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Минимальный пример»: ilustra la estructura de 5 slots, no un caso de florería; vale para todo prompt</t>
-        </is>
-      </c>
-      <c r="TC10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11684,14 +11571,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ11" s="4" t="inlineStr"/>
-      <c r="TA11" s="4" t="inlineStr"/>
-      <c r="TB11" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Anti-Slop Rules»; las reglas son 002340–002346</t>
-        </is>
-      </c>
-      <c r="TC11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13217,18 +13096,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ12" s="4" t="inlineStr"/>
-      <c r="TA12" s="4" t="inlineStr">
-        <is>
-          <t>sin elogios vagos</t>
-        </is>
-      </c>
-      <c r="TB12" s="4" t="inlineStr">
-        <is>
-          <t>«Vague praise = деградация результата»</t>
-        </is>
-      </c>
-      <c r="TC12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13244,14 +13111,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ13" s="4" t="inlineStr"/>
-      <c r="TA13" s="4" t="inlineStr"/>
-      <c r="TB13" s="4" t="inlineStr">
-        <is>
-          <t>cabecera de tabla «No escribas | Escribe»; las filas son 002343–002346</t>
-        </is>
-      </c>
-      <c r="TC13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13267,14 +13126,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ14" s="4" t="inlineStr"/>
-      <c r="TA14" s="4" t="inlineStr"/>
-      <c r="TB14" s="4" t="inlineStr">
-        <is>
-          <t>separador de tabla markdown</t>
-        </is>
-      </c>
-      <c r="TC14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -14825,18 +14676,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ15" s="4" t="inlineStr"/>
-      <c r="TA15" s="4" t="inlineStr">
-        <is>
-          <t>prohibido: stunning, incredible, epic, gorgeous, masterpiece → escribir hechos visuales: overcast daylight, brushed aluminum, chipped paint, 50mm feel</t>
-        </is>
-      </c>
-      <c r="TB15" s="4" t="inlineStr">
-        <is>
-          <t>fila de la tabla «Не пиши | Пиши»; aplica a todo prompt de GPT Image 2</t>
-        </is>
-      </c>
-      <c r="TC15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -16387,18 +16226,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ16" s="4" t="inlineStr"/>
-      <c r="TA16" s="4" t="inlineStr">
-        <is>
-          <t>prohibidas etiquetas de estilo («minimalist brutalist luxury photoreal») → atributos visibles: «cream background, heavy black sans-serif, asymmetrical type block, one hero object, generous negative space»</t>
-        </is>
-      </c>
-      <c r="TB16" s="4" t="inlineStr">
-        <is>
-          <t>fila de la tabla «Не пиши | Пиши»</t>
-        </is>
-      </c>
-      <c r="TC16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -17934,18 +17761,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ17" s="4" t="inlineStr"/>
-      <c r="TA17" s="4" t="inlineStr">
-        <is>
-          <t>prohibido «como en un anuncio de Apple» → hechos visuales concretos</t>
-        </is>
-      </c>
-      <c r="TB17" s="4" t="inlineStr">
-        <is>
-          <t>fila de la tabla «Не пиши | Пиши»</t>
-        </is>
-      </c>
-      <c r="TC17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -19491,18 +19306,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ18" s="4" t="inlineStr"/>
-      <c r="TA18" s="4" t="inlineStr">
-        <is>
-          <t>prohibido lenguaje de ambiente que oculta requisitos → enunciado directo: «image must contain a transit kiosk»</t>
-        </is>
-      </c>
-      <c r="TB18" s="4" t="inlineStr">
-        <is>
-          <t>fila de la tabla «Не пиши | Пиши»</t>
-        </is>
-      </c>
-      <c r="TC18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -19518,14 +19321,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ19" s="4" t="inlineStr"/>
-      <c r="TA19" s="4" t="inlineStr"/>
-      <c r="TB19" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Quality Settings»; las reglas son 002350–002353</t>
-        </is>
-      </c>
-      <c r="TC19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -19541,14 +19336,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ20" s="4" t="inlineStr"/>
-      <c r="TA20" s="4" t="inlineStr"/>
-      <c r="TB20" s="4" t="inlineStr">
-        <is>
-          <t>cabecera de tabla «Setting | Cuándo»</t>
-        </is>
-      </c>
-      <c r="TC20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -19564,14 +19351,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ21" s="4" t="inlineStr"/>
-      <c r="TA21" s="4" t="inlineStr"/>
-      <c r="TB21" s="4" t="inlineStr">
-        <is>
-          <t>separador de tabla markdown</t>
-        </is>
-      </c>
-      <c r="TC21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -21082,18 +20861,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ22" s="4" t="inlineStr"/>
-      <c r="TA22" s="4" t="inlineStr">
-        <is>
-          <t>quality: low</t>
-        </is>
-      </c>
-      <c r="TB22" s="4" t="inlineStr">
-        <is>
-          <t>«quality: low | High-volume, превью, exploratory, latency-sensitive, draft»: corresponde al paso de borradores</t>
-        </is>
-      </c>
-      <c r="TC22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -22629,18 +22396,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ23" s="4" t="inlineStr"/>
-      <c r="TA23" s="4" t="inlineStr">
-        <is>
-          <t>quality: medium como punto de partida</t>
-        </is>
-      </c>
-      <c r="TB23" s="4" t="inlineStr">
-        <is>
-          <t>«quality: medium | Default starting point»; choca con 002353. Decisión de Eric (C1): quality la elige el usuario y esta línea se le muestra como opción</t>
-        </is>
-      </c>
-      <c r="TC23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -24171,22 +23926,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ24" s="4" t="inlineStr">
-        <is>
-          <t>A1: F32: texto extenso o pequeño | A2: F04: infografía o diagrama, retrato, identidad de marca | A3: F10: edición de imagen existente (T5) + F20: todas, solo los héroes</t>
-        </is>
-      </c>
-      <c r="TA24" s="4" t="inlineStr">
-        <is>
-          <t>quality: high | quality: high | quality: high</t>
-        </is>
-      </c>
-      <c r="TB24" s="4" t="inlineStr">
-        <is>
-          <t>«Маленький/плотный текст» → texto pequeño o denso | «infographics, портреты, brand assets» → tipo de pieza infografía, retrato, identidad de marca | «identity-sensitive edits» → edición con identidad de personas a conservar</t>
-        </is>
-      </c>
-      <c r="TC24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -25712,18 +25451,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ25" s="4" t="inlineStr"/>
-      <c r="TA25" s="4" t="inlineStr">
-        <is>
-          <t>empezar con quality: low y subir si hace falta</t>
-        </is>
-      </c>
-      <c r="TB25" s="4" t="inlineStr">
-        <is>
-          <t>«Стартуй с low, апгрейди по необходимости»; choca con 002351. Decisión de Eric (C1): quality la elige el usuario y esta línea se le muestra como opción</t>
-        </is>
-      </c>
-      <c r="TC25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -25739,14 +25466,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ26" s="4" t="inlineStr"/>
-      <c r="TA26" s="4" t="inlineStr"/>
-      <c r="TB26" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Tamaños (gpt-image-2)»; las reglas son 002355–002365</t>
-        </is>
-      </c>
-      <c r="TC26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -27282,18 +27001,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ27" s="4" t="inlineStr"/>
-      <c r="TA27" s="4" t="inlineStr">
-        <is>
-          <t>lado mayor &lt; 3840 px</t>
-        </is>
-      </c>
-      <c r="TB27" s="4" t="inlineStr">
-        <is>
-          <t>«Max edge: &lt;3840px»</t>
-        </is>
-      </c>
-      <c r="TC27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -28829,18 +28536,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ28" s="4" t="inlineStr"/>
-      <c r="TA28" s="4" t="inlineStr">
-        <is>
-          <t>ambos lados múltiplos de 16</t>
-        </is>
-      </c>
-      <c r="TB28" s="4" t="inlineStr">
-        <is>
-          <t>«Обе стороны: кратны 16»</t>
-        </is>
-      </c>
-      <c r="TC28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -30376,18 +30071,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ29" s="4" t="inlineStr"/>
-      <c r="TA29" s="4" t="inlineStr">
-        <is>
-          <t>relación de aspecto máxima 3:1</t>
-        </is>
-      </c>
-      <c r="TB29" s="4" t="inlineStr">
-        <is>
-          <t>«Aspect ratio: max 3:1 (long:short)»</t>
-        </is>
-      </c>
-      <c r="TC29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -31923,18 +31606,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ30" s="4" t="inlineStr"/>
-      <c r="TA30" s="4" t="inlineStr">
-        <is>
-          <t>total de píxeles entre 655 360 y 8 294 400</t>
-        </is>
-      </c>
-      <c r="TB30" s="4" t="inlineStr">
-        <is>
-          <t>«Total pixels: 655 360 – 8 294 400»</t>
-        </is>
-      </c>
-      <c r="TC30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -33470,18 +33141,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ31" s="4" t="inlineStr"/>
-      <c r="TA31" s="4" t="inlineStr">
-        <is>
-          <t>límite fiable 2560×1440</t>
-        </is>
-      </c>
-      <c r="TB31" s="4" t="inlineStr">
-        <is>
-          <t>«Reliable upper bound: 2560×1440»</t>
-        </is>
-      </c>
-      <c r="TC31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -33497,14 +33156,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ32" s="4" t="inlineStr"/>
-      <c r="TA32" s="4" t="inlineStr"/>
-      <c r="TB32" s="4" t="inlineStr">
-        <is>
-          <t>rótulo «Habituales:» que introduce la lista 002361–002364</t>
-        </is>
-      </c>
-      <c r="TC32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -34970,18 +34621,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ33" s="4" t="inlineStr"/>
-      <c r="TA33" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="TB33" s="4" t="inlineStr">
-        <is>
-          <t>«Portrait 1024×1536» = 2:3</t>
-        </is>
-      </c>
-      <c r="TC33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -36447,18 +36086,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ34" s="4" t="inlineStr"/>
-      <c r="TA34" s="4" t="inlineStr">
-        <is>
-          <t>1536×1024</t>
-        </is>
-      </c>
-      <c r="TB34" s="4" t="inlineStr">
-        <is>
-          <t>«Landscape 1536×1024» = 3:2</t>
-        </is>
-      </c>
-      <c r="TC34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -37924,18 +37551,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ35" s="4" t="inlineStr"/>
-      <c r="TA35" s="4" t="inlineStr">
-        <is>
-          <t>1024×1024</t>
-        </is>
-      </c>
-      <c r="TB35" s="4" t="inlineStr">
-        <is>
-          <t>«Square 1024×1024» = 1:1</t>
-        </is>
-      </c>
-      <c r="TC35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -39391,18 +39006,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ36" s="4" t="inlineStr"/>
-      <c r="TA36" s="4" t="inlineStr">
-        <is>
-          <t>2560×1440</t>
-        </is>
-      </c>
-      <c r="TB36" s="4" t="inlineStr">
-        <is>
-          <t>«2K 2560×1440» = 16:9 a 2K</t>
-        </is>
-      </c>
-      <c r="TC36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -40903,18 +40506,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ37" s="4" t="inlineStr"/>
-      <c r="TA37" s="4" t="inlineStr">
-        <is>
-          <t>1:8 y 8:1 no se hacen con GPT Image 2: cambiar a Nano Banana</t>
-        </is>
-      </c>
-      <c r="TB37" s="4" t="inlineStr">
-        <is>
-          <t>«Экстрим вроде 1:8 / 8:1 GPT Image 2 НЕ умеет — иди в Nano Banana»</t>
-        </is>
-      </c>
-      <c r="TC37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -40930,14 +40521,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ38" s="4" t="inlineStr"/>
-      <c r="TA38" s="4" t="inlineStr"/>
-      <c r="TB38" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Text in Image»; las reglas son 002367–002372</t>
-        </is>
-      </c>
-      <c r="TC38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -42468,18 +42051,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ39" s="4" t="inlineStr"/>
-      <c r="TA39" s="4" t="inlineStr">
-        <is>
-          <t>texto literal entre "..." o en MAYÚSCULAS</t>
-        </is>
-      </c>
-      <c r="TB39" s="4" t="inlineStr">
-        <is>
-          <t>sección «Text in Image»: «Литеральный текст в "..." или ALL CAPS»</t>
-        </is>
-      </c>
-      <c r="TC39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -44005,18 +43576,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ40" s="4" t="inlineStr"/>
-      <c r="TA40" s="4" t="inlineStr">
-        <is>
-          <t>fuente, tamaño, color y posición del texto, explícitos</t>
-        </is>
-      </c>
-      <c r="TB40" s="4" t="inlineStr">
-        <is>
-          <t>«Шрифт, размер, цвет, позиция — явно»</t>
-        </is>
-      </c>
-      <c r="TC40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -45537,18 +45096,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ41" s="4" t="inlineStr"/>
-      <c r="TA41" s="4" t="inlineStr">
-        <is>
-          <t>palabras difíciles y marcas deletreadas letra por letra</t>
-        </is>
-      </c>
-      <c r="TB41" s="4" t="inlineStr">
-        <is>
-          <t>«Сложные слова и бренды: спеллинг по буквам»</t>
-        </is>
-      </c>
-      <c r="TC41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -47069,18 +46616,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ42" s="4" t="inlineStr"/>
-      <c r="TA42" s="4" t="inlineStr">
-        <is>
-          <t>no extra words, no duplicate text, no watermarks</t>
-        </is>
-      </c>
-      <c r="TB42" s="4" t="inlineStr">
-        <is>
-          <t>«Защита от мусора: no extra words, no duplicate text, no watermarks»</t>
-        </is>
-      </c>
-      <c r="TC42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -48596,18 +48131,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ43" s="4" t="inlineStr"/>
-      <c r="TA43" s="4" t="inlineStr">
-        <is>
-          <t>100 percent readable and physically believable</t>
-        </is>
-      </c>
-      <c r="TB43" s="4" t="inlineStr">
-        <is>
-          <t>«Для нечитаемого мелкого текста: 100 percent readable…»</t>
-        </is>
-      </c>
-      <c r="TC43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -50128,18 +49651,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ44" s="4" t="inlineStr"/>
-      <c r="TA44" s="4" t="inlineStr">
-        <is>
-          <t>quality: high obligatorio</t>
-        </is>
-      </c>
-      <c r="TB44" s="4" t="inlineStr">
-        <is>
-          <t>«Маленький/плотный/multi-font → quality: high обязательно»</t>
-        </is>
-      </c>
-      <c r="TC44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -50155,14 +49666,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ45" s="4" t="inlineStr"/>
-      <c r="TA45" s="4" t="inlineStr"/>
-      <c r="TB45" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Editing — lógica de dos columnas»; el contenido está en 002374–002385</t>
-        </is>
-      </c>
-      <c r="TC45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -51533,18 +51036,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ46" s="4" t="inlineStr"/>
-      <c r="TA46" s="4" t="inlineStr">
-        <is>
-          <t>openai/gpt-image-2/edit (fal.ai) o el equivalente de la API de OpenAI</t>
-        </is>
-      </c>
-      <c r="TB46" s="4" t="inlineStr">
-        <is>
-          <t>«Endpoint: openai/gpt-image-2/edit (на fal.ai)…»; la ejecución la hace el usuario</t>
-        </is>
-      </c>
-      <c r="TC46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -52920,18 +52411,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ47" s="4" t="inlineStr"/>
-      <c r="TA47" s="4" t="inlineStr">
-        <is>
-          <t>Change: [single concrete change] / Preserve: face, identity, pose, lighting, framing, background, geometry, text, layout / Constraints: no extra objects, no redesign, no drift</t>
-        </is>
-      </c>
-      <c r="TB47" s="4" t="inlineStr">
-        <is>
-          <t>bloque literal bajo «Editing — двухколоночная логика»</t>
-        </is>
-      </c>
-      <c r="TC47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -52947,14 +52426,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ48" s="4" t="inlineStr"/>
-      <c r="TA48" s="4" t="inlineStr"/>
-      <c r="TB48" s="4" t="inlineStr">
-        <is>
-          <t>rótulo «Reglas de edit:» que introduce 002377–002380</t>
-        </is>
-      </c>
-      <c r="TC48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -54320,18 +53791,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ49" s="4" t="inlineStr"/>
-      <c r="TA49" s="4" t="inlineStr">
-        <is>
-          <t>un solo cambio por iteración</t>
-        </is>
-      </c>
-      <c r="TB49" s="4" t="inlineStr">
-        <is>
-          <t>«Один edit за итерацию»</t>
-        </is>
-      </c>
-      <c r="TC49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -55712,18 +55171,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ50" s="4" t="inlineStr"/>
-      <c r="TA50" s="4" t="inlineStr">
-        <is>
-          <t>lista Preserve completa en cada iteración</t>
-        </is>
-      </c>
-      <c r="TB50" s="4" t="inlineStr">
-        <is>
-          <t>«Preserve list повторять каждую итерацию. Иначе дрейф»</t>
-        </is>
-      </c>
-      <c r="TC50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -57109,18 +56556,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ51" s="4" t="inlineStr"/>
-      <c r="TA51" s="4" t="inlineStr">
-        <is>
-          <t>enumerar lo que NO se toca (saturación, contraste, layout, flechas, etiquetas, ángulo de cámara)</t>
-        </is>
-      </c>
-      <c r="TB51" s="4" t="inlineStr">
-        <is>
-          <t>«Surgical edits: явно перечисли что НЕ трогать…»; el contenido depende de cada edición</t>
-        </is>
-      </c>
-      <c r="TC51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -58491,18 +57926,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ52" s="4" t="inlineStr"/>
-      <c r="TA52" s="4" t="inlineStr">
-        <is>
-          <t>mask_image_url para ediciones puntuales</t>
-        </is>
-      </c>
-      <c r="TB52" s="4" t="inlineStr">
-        <is>
-          <t>«Опционально: mask_image_url для точечных edits»</t>
-        </is>
-      </c>
-      <c r="TC52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -58518,14 +57941,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ53" s="4" t="inlineStr"/>
-      <c r="TA53" s="4" t="inlineStr"/>
-      <c r="TB53" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Patrones de edición»; los patrones son 002382–002385</t>
-        </is>
-      </c>
-      <c r="TC53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -59881,18 +59296,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ54" s="4" t="inlineStr"/>
-      <c r="TA54" s="4" t="inlineStr">
-        <is>
-          <t>Change garments only. Preserve exact face, body shape, pose, hair, expression, background, camera angle. Match lighting/shadows so outfit looks naturally worn.</t>
-        </is>
-      </c>
-      <c r="TB54" s="4" t="inlineStr">
-        <is>
-          <t>patrón «Virtual try-on» → subtipo «edición: cambiar vestuario» (aprobado por Eric, consulta C2)</t>
-        </is>
-      </c>
-      <c r="TC54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -61343,22 +60746,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ55" s="4" t="inlineStr">
-        <is>
-          <t>A1: F10: edición: quitar objeto | A2: F10: edición: quitar objeto | A3: F10: edición: quitar objeto</t>
-        </is>
-      </c>
-      <c r="TA55" s="4" t="inlineStr">
-        <is>
-          <t>Remove [X]. Do not change anything else. | no enviar input_fidelity a gpt-image-2 (alta fidelidad por defecto) | input_fidelity: high</t>
-        </is>
-      </c>
-      <c r="TB55" s="4" t="inlineStr">
-        <is>
-          <t>patrón «Object removal», parte válida en GPT Image 2 | «(только gpt-image-1.5/1, в gpt-image-2 high-fidelity по умолчанию)» | «Use input_fidelity: high… (только gpt-image-1.5/1)»</t>
-        </is>
-      </c>
-      <c r="TC55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -62739,18 +62126,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ56" s="4" t="inlineStr"/>
-      <c r="TA56" s="4" t="inlineStr">
-        <is>
-          <t>Change ONLY environmental conditions: lighting direction/quality, shadows, atmosphere, precipitation. Preserve identity, geometry, camera angle, object placement.</t>
-        </is>
-      </c>
-      <c r="TB56" s="4" t="inlineStr">
-        <is>
-          <t>patrón «Lighting/weather swap»</t>
-        </is>
-      </c>
-      <c r="TC56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -64101,18 +63476,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ57" s="4" t="inlineStr"/>
-      <c r="TA57" s="4" t="inlineStr">
-        <is>
-          <t>Swap [furniture]. Preserve camera angle, lighting, shadows, surrounding context. Photorealistic contact shadows.</t>
-        </is>
-      </c>
-      <c r="TB57" s="4" t="inlineStr">
-        <is>
-          <t>patrón «Interior swap» → subtipo «edición: cambiar mobiliario u objeto» (aprobado, consulta C2); «Photorealistic» choca con la prohibición de esa palabra por Eric (templates §1): se conserva el efecto con atributos visibles</t>
-        </is>
-      </c>
-      <c r="TC57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -65623,18 +64986,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ58" s="4" t="inlineStr"/>
-      <c r="TA58" s="4" t="inlineStr">
-        <is>
-          <t>hasta 16 imágenes de referencia</t>
-        </is>
-      </c>
-      <c r="TB58" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Multi-Image — до 16 рефов»: lleva el límite de referencias</t>
-        </is>
-      </c>
-      <c r="TC58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -67150,18 +66501,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ59" s="4" t="inlineStr"/>
-      <c r="TA59" s="4" t="inlineStr">
-        <is>
-          <t>cada referencia indexada con su rol: «Image N: rol»</t>
-        </is>
-      </c>
-      <c r="TB59" s="4" t="inlineStr">
-        <is>
-          <t>«Индексируй с ролью, не только номером»</t>
-        </is>
-      </c>
-      <c r="TC59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -68667,18 +68006,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ60" s="4" t="inlineStr"/>
-      <c r="TA60" s="4" t="inlineStr">
-        <is>
-          <t>Image 1: base scene / Image 2: jacket reference (apply only…) / Image 3: lighting reference (apply…)</t>
-        </is>
-      </c>
-      <c r="TB60" s="4" t="inlineStr">
-        <is>
-          <t>ejemplo del indexado con rol</t>
-        </is>
-      </c>
-      <c r="TC60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -68694,14 +68021,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ61" s="4" t="inlineStr"/>
-      <c r="TA61" s="4" t="inlineStr"/>
-      <c r="TB61" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Style Transfer»; la regla es 002390</t>
-        </is>
-      </c>
-      <c r="TC61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -70042,18 +69361,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ62" s="4" t="inlineStr"/>
-      <c r="TA62" s="4" t="inlineStr">
-        <is>
-          <t>nada de «minimalist», «editorial»: nombrar paleta, tratamiento de bordes, silueta, sombras y lógica de planos de la referencia</t>
-        </is>
-      </c>
-      <c r="TB62" s="4" t="inlineStr">
-        <is>
-          <t>sección «Style Transfer»</t>
-        </is>
-      </c>
-      <c r="TC62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -70069,14 +69376,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ63" s="4" t="inlineStr"/>
-      <c r="TA63" s="4" t="inlineStr"/>
-      <c r="TB63" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «World Knowledge»; la regla es 002392</t>
-        </is>
-      </c>
-      <c r="TC63" s="4" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -71542,18 +70841,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ64" s="4" t="inlineStr"/>
-      <c r="TA64" s="4" t="inlineStr">
-        <is>
-          <t>dar el ancla histórica o cultural (p. ej. «Bethel, NY, August 1969») en vez de describir cada detalle</t>
-        </is>
-      </c>
-      <c r="TB64" s="4" t="inlineStr">
-        <is>
-          <t>sección «World Knowledge»</t>
-        </is>
-      </c>
-      <c r="TC64" s="4" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -71569,14 +70856,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ65" s="4" t="inlineStr"/>
-      <c r="TA65" s="4" t="inlineStr"/>
-      <c r="TB65" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Iteration Strategy»; las reglas son 002394–002397</t>
-        </is>
-      </c>
-      <c r="TC65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -73082,18 +72361,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ66" s="4" t="inlineStr"/>
-      <c r="TA66" s="4" t="inlineStr">
-        <is>
-          <t>el primer prompt es limpio, sin acumulaciones</t>
-        </is>
-      </c>
-      <c r="TB66" s="4" t="inlineStr">
-        <is>
-          <t>«Стартуй с чистого базового промпта»</t>
-        </is>
-      </c>
-      <c r="TC66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -74614,18 +73881,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ67" s="4" t="inlineStr"/>
-      <c r="TA67" s="4" t="inlineStr">
-        <is>
-          <t>un cambio por ronda («Make lighting warmer», «remove extra tree», «restore original background»)</t>
-        </is>
-      </c>
-      <c r="TB67" s="4" t="inlineStr">
-        <is>
-          <t>«Один change за раунд»</t>
-        </is>
-      </c>
-      <c r="TC67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -76136,18 +75391,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ68" s="4" t="inlineStr"/>
-      <c r="TA68" s="4" t="inlineStr">
-        <is>
-          <t>si hay deriva, volver a enumerar los invariantes</t>
-        </is>
-      </c>
-      <c r="TB68" s="4" t="inlineStr">
-        <is>
-          <t>«При drift — перечисли invariants заново»</t>
-        </is>
-      </c>
-      <c r="TC68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -77673,18 +76916,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ69" s="4" t="inlineStr"/>
-      <c r="TA69" s="4" t="inlineStr">
-        <is>
-          <t>prompts largos en secciones con etiqueta</t>
-        </is>
-      </c>
-      <c r="TB69" s="4" t="inlineStr">
-        <is>
-          <t>«Для длинных промптов — labeled sections»</t>
-        </is>
-      </c>
-      <c r="TC69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -77700,14 +76931,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ70" s="4" t="inlineStr"/>
-      <c r="TA70" s="4" t="inlineStr"/>
-      <c r="TB70" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Use-Case Templates»; las plantillas son 002400–002408</t>
-        </is>
-      </c>
-      <c r="TC70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -77723,14 +76946,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ71" s="4" t="inlineStr"/>
-      <c r="TA71" s="4" t="inlineStr"/>
-      <c r="TB71" s="4" t="inlineStr">
-        <is>
-          <t>encabezado de la plantilla «Photoreal Editorial» (002400)</t>
-        </is>
-      </c>
-      <c r="TC71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -79121,18 +78336,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ72" s="4" t="inlineStr"/>
-      <c r="TA72" s="4" t="inlineStr">
-        <is>
-          <t>Use Case: editorial photograph, looks like a real photo / Constraints: no glamorization, no heavy retouching, no studio gloss (+ Scene/Subject/Important Details a llenar)</t>
-        </is>
-      </c>
-      <c r="TB72" s="4" t="inlineStr">
-        <is>
-          <t>plantilla «Photoreal Editorial» (biblioteca)</t>
-        </is>
-      </c>
-      <c r="TC72" s="4" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -79148,14 +78351,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ73" s="4" t="inlineStr"/>
-      <c r="TA73" s="4" t="inlineStr"/>
-      <c r="TB73" s="4" t="inlineStr">
-        <is>
-          <t>encabezado de la plantilla «Product Mockup» (002402)</t>
-        </is>
-      </c>
-      <c r="TC73" s="4" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -80351,18 +79546,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ74" s="4" t="inlineStr"/>
-      <c r="TA74" s="4" t="inlineStr">
-        <is>
-          <t>Scene: plain white opaque background / Important Details: crisp silhouette, no halos/fringing, light contact shadow, preserve label legibility exactly, preserve geometry / Use Case: product mockup / Constraints: no restyling, only background removal + light polish</t>
-        </is>
-      </c>
-      <c r="TB74" s="4" t="inlineStr">
-        <is>
-          <t>plantilla «Product Mockup»: «preserve label… only background removal» supone foto de producto de referencia</t>
-        </is>
-      </c>
-      <c r="TC74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -80378,14 +79561,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ75" s="4" t="inlineStr"/>
-      <c r="TA75" s="4" t="inlineStr"/>
-      <c r="TB75" s="4" t="inlineStr">
-        <is>
-          <t>encabezado de la plantilla «UI Mockup» (002404)</t>
-        </is>
-      </c>
-      <c r="TC75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -81811,18 +80986,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ76" s="4" t="inlineStr"/>
-      <c r="TA76" s="4" t="inlineStr">
-        <is>
-          <t>Subject: … describe AS IF IT EXISTS, not concept art / Important Details: exact copy in quotes… / Use Case: shipped product screenshot / Constraints: no sketch language, no placeholder text, no Lorem Ipsum / Quality: high</t>
-        </is>
-      </c>
-      <c r="TB76" s="4" t="inlineStr">
-        <is>
-          <t>plantilla «UI Mockup»</t>
-        </is>
-      </c>
-      <c r="TC76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -81838,14 +81001,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ77" s="4" t="inlineStr"/>
-      <c r="TA77" s="4" t="inlineStr"/>
-      <c r="TB77" s="4" t="inlineStr">
-        <is>
-          <t>encabezado de la plantilla «Marketing Creative with Text» (002406)</t>
-        </is>
-      </c>
-      <c r="TC77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -83286,18 +82441,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ78" s="4" t="inlineStr"/>
-      <c r="TA78" s="4" t="inlineStr">
-        <is>
-          <t>Use Case: ad creative for [audience] / Text: "EXACT HEADLINE" in [font], [color], [position] / Constraints: no extra text, no duplicate text, no watermarks, no unrelated logos / Quality: high</t>
-        </is>
-      </c>
-      <c r="TB78" s="4" t="inlineStr">
-        <is>
-          <t>plantilla «Marketing Creative with Text»</t>
-        </is>
-      </c>
-      <c r="TC78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -83313,14 +82456,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ79" s="4" t="inlineStr"/>
-      <c r="TA79" s="4" t="inlineStr"/>
-      <c r="TB79" s="4" t="inlineStr">
-        <is>
-          <t>encabezado de la plantilla «Infographic / Diagram» (002408)</t>
-        </is>
-      </c>
-      <c r="TC79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -84681,18 +83816,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ80" s="4" t="inlineStr"/>
-      <c r="TA80" s="4" t="inlineStr">
-        <is>
-          <t>Title: "[TITLE]" / Content flow / Visual format / Use Case: educational infographic for [audience] / Constraints: readable labels at all sizes, clear hierarchy, no clutter, no decorative noise, ample whitespace / Quality: high / Size: 1536×1024</t>
-        </is>
-      </c>
-      <c r="TB80" s="4" t="inlineStr">
-        <is>
-          <t>plantilla «Infographic / Diagram»; sus etiquetas Title/Content flow/Visual format no son los 5 slots: según templates §6 se usan como módulo dentro de los 5 slots</t>
-        </is>
-      </c>
-      <c r="TC80" s="4" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -84708,14 +83831,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ81" s="4" t="inlineStr"/>
-      <c r="TA81" s="4" t="inlineStr"/>
-      <c r="TB81" s="4" t="inlineStr">
-        <is>
-          <t>encabezado «Migration from Older GPT-Image»; las reglas son 002410–002412</t>
-        </is>
-      </c>
-      <c r="TC81" s="4" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -86231,18 +85346,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ82" s="4" t="inlineStr"/>
-      <c r="TA82" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="TB82" s="4" t="inlineStr">
-        <is>
-          <t>«Промпты в основном переносятся как есть»: migración de versión de modelo (decisión de Eric, C3)</t>
-        </is>
-      </c>
-      <c r="TC82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -87748,18 +86851,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ83" s="4" t="inlineStr"/>
-      <c r="TA83" s="4" t="inlineStr">
-        <is>
-          <t>tras migrar, revisar calidad, latencia y tasa de reintentos; reajustar</t>
-        </is>
-      </c>
-      <c r="TB83" s="4" t="inlineStr">
-        <is>
-          <t>«После переноса — посмотри качество, latency, retry-rate»: migración de versión de modelo (decisión de Eric, C3)</t>
-        </is>
-      </c>
-      <c r="TC83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -89290,18 +88381,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ84" s="4" t="inlineStr"/>
-      <c r="TA84" s="4" t="inlineStr">
-        <is>
-          <t>gpt-image-1-mini solo para bajar costo de lotes de bajo riesgo</t>
-        </is>
-      </c>
-      <c r="TB84" s="4" t="inlineStr">
-        <is>
-          <t>«gpt-image-1-mini — только если главное снизить цену batch'а»</t>
-        </is>
-      </c>
-      <c r="TC84" s="4" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -89317,14 +88396,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ85" s="4" t="inlineStr"/>
-      <c r="TA85" s="4" t="inlineStr"/>
-      <c r="TB85" s="4" t="inlineStr">
-        <is>
-          <t>separador horizontal markdown antes de la atribución</t>
-        </is>
-      </c>
-      <c r="TC85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -89340,14 +88411,6 @@
           <t>X</t>
         </is>
       </c>
-      <c r="SZ86" s="4" t="inlineStr"/>
-      <c r="TA86" s="4" t="inlineStr"/>
-      <c r="TB86" s="4" t="inlineStr">
-        <is>
-          <t>atribución de autor y licencia CC BY 4.0; se conserva en la traza de fuentes (templates §11), no regula el prompt</t>
-        </is>
-      </c>
-      <c r="TC86" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -89360,268 +88423,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Clasificación desde cero de los 84 textos de skills/image/references/gpt-image.md (base original 13,005).</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Criterios fijos (escritos también en la hoja "criterios" del Excel):</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>- Una fila por aplicación (§7.2: una condición alternativa son dos aplicaciones del mismo texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>- Faceta no mencionada en `r` (restricciones) = el texto no la restringe: X en todos sus valores.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>- F01 siempre "5 Imagen". P01 (flujo): todos. F02 (paso): el que indique la fila; por defecto los pasos donde se</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  redacta un prompt de imagen (E5.2–E5.6).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>- Uso operativo (§5.3): ningún template está verificado todavía, así que nada es "INCORPORADA A TEMPLATE";</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  lo que se mecaniza en el template (estructura, parámetros, reglas universales) es "APLICACIÓN EN CONSTRUCCIÓN</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  DE TEMPLATE"; lo que depende del contenido del caso es "ACTIVO EN SELECCIÓN"; ejemplos y revisiones son</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  "APLICACIÓN EN CONTROL O ENTREGA".</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>- Objeto regulado: lo que se ve en la imagen → activo visual o sonoro; estructura del prompt y parámetros →</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  campo o esquema; proceso de generación e iteración → registro de ejecución (run).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>- Acción al activarse (§1.13 + instrucción de Eric 2026-10-23): agregar al prompt · seleccionar estructura · fijar</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  parámetro · validar el prompt · validar contra el ejemplo · excluir del prompt · solo traza.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>- Origen de evidencia: «Evidencia directa» (texto literal de un skill instalado). Evidencia de la afirmación:</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  «Afirmación fuente por contrastar» salvo conflicto entre fuentes. Adopción: «adopción documental».</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>- Unidad de las filas de activo visual: «imagen fija suelta» (extensión aprobada por Eric el 2026-10-23, respuesta a</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  la consulta U1).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>matriz_eric.py: matriz en el formato pedido por Eric (2026-10-24), para cualquier archivo clasificado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>- Sin textos en la matriz (instrucción de Eric): columna A = número del texto (id persistente de la base de 13,005</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  textos originales), columna B = línea del archivo. El texto se localiza en la base por ese número.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>- Una fila por texto. Si el texto tiene casos alternativos (§7.2), sus X van en la misma fila y la columna "casos"</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  dice qué valores se combinan en cada caso.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>- Columnas de lo general a lo particular: tipo de texto → imagen o video → modelo → universal → interno o externo →</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  tipo de pieza → sujeto → número de personas → resto de facetas → proceso → atributos → acción, destino, valor</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  a insertar y fundamento al final.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>- Antes de escribir corre la verificación de la clasificación; después reabre el Excel y comprueba el formato y que</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  los números sean exactamente los textos del archivo en la base, sin faltantes ni repetidos. Si algo falla, sale</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  con error.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    python3 matriz_eric.py &lt;carpeta_con_clasificacion.py&gt; &lt;archivo_fuente&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>código</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>pregunta</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:C518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>